<commit_message>
Data export W14-2026 (2026-04-06T17:44:44Z)
</commit_message>
<xml_diff>
--- a/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
+++ b/files/power_outage_area/Power_Cuts_2026_Area_Summary.xlsx
@@ -643,22 +643,22 @@
         </is>
       </c>
       <c r="C2" s="9" t="n">
-        <v>34371</v>
+        <v>38444</v>
       </c>
       <c r="D2" s="9" t="n">
-        <v>47.39716204476192</v>
+        <v>47.07985843222259</v>
       </c>
       <c r="E2" s="9" t="inlineStr"/>
       <c r="F2" s="9" t="inlineStr">
         <is>
-          <t>61546:00:00</t>
+          <t>70840:00:00</t>
         </is>
       </c>
       <c r="G2" s="9" t="n">
-        <v>61546</v>
+        <v>70840</v>
       </c>
       <c r="H2" s="9" t="n">
-        <v>47.57215514709293</v>
+        <v>47.05257214971273</v>
       </c>
     </row>
     <row r="3">
@@ -673,22 +673,22 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>15896</v>
+        <v>17719</v>
       </c>
       <c r="D3" s="10" t="n">
-        <v>21.92037729084215</v>
+        <v>21.69930318282572</v>
       </c>
       <c r="E3" s="10" t="inlineStr"/>
       <c r="F3" s="10" t="inlineStr">
         <is>
-          <t>26256:00:00</t>
+          <t>30854:00:00</t>
         </is>
       </c>
       <c r="G3" s="10" t="n">
-        <v>26256</v>
+        <v>30854</v>
       </c>
       <c r="H3" s="10" t="n">
-        <v>20.29464962048016</v>
+        <v>20.49350735611571</v>
       </c>
     </row>
     <row r="4">
@@ -703,22 +703,22 @@
         </is>
       </c>
       <c r="C4" s="11" t="n">
-        <v>22250</v>
+        <v>25494</v>
       </c>
       <c r="D4" s="11" t="n">
-        <v>30.68246066439593</v>
+        <v>31.22083838495169</v>
       </c>
       <c r="E4" s="11" t="inlineStr"/>
       <c r="F4" s="11" t="inlineStr">
         <is>
-          <t>41572:00:00</t>
+          <t>48861:00:00</t>
         </is>
       </c>
       <c r="G4" s="11" t="n">
-        <v>41572</v>
+        <v>48861</v>
       </c>
       <c r="H4" s="11" t="n">
-        <v>32.13319523242692</v>
+        <v>32.45392049417157</v>
       </c>
     </row>
   </sheetData>
@@ -1103,7 +1103,7 @@
         <v>3762</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0</v>
+        <v>4073</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0</v>
@@ -1266,7 +1266,7 @@
         <v>1445</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>0</v>
+        <v>1823</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>0</v>
@@ -1429,7 +1429,7 @@
         <v>2211</v>
       </c>
       <c r="O4" s="11" t="n">
-        <v>0</v>
+        <v>3244</v>
       </c>
       <c r="P4" s="11" t="n">
         <v>0</v>
@@ -1592,7 +1592,7 @@
         <v>7418</v>
       </c>
       <c r="O5" s="12" t="n">
-        <v>0</v>
+        <v>9140</v>
       </c>
       <c r="P5" s="12" t="n">
         <v>0</v>
@@ -2091,7 +2091,7 @@
         <v>7619</v>
       </c>
       <c r="O2" s="9" t="n">
-        <v>0</v>
+        <v>9294</v>
       </c>
       <c r="P2" s="9" t="n">
         <v>0</v>
@@ -2254,7 +2254,7 @@
         <v>3146</v>
       </c>
       <c r="O3" s="10" t="n">
-        <v>0</v>
+        <v>4598</v>
       </c>
       <c r="P3" s="10" t="n">
         <v>0</v>
@@ -2417,7 +2417,7 @@
         <v>4157</v>
       </c>
       <c r="O4" s="11" t="n">
-        <v>0</v>
+        <v>7289</v>
       </c>
       <c r="P4" s="11" t="n">
         <v>0</v>
@@ -2580,7 +2580,7 @@
         <v>14922</v>
       </c>
       <c r="O5" s="12" t="n">
-        <v>0</v>
+        <v>21181</v>
       </c>
       <c r="P5" s="12" t="n">
         <v>0</v>
@@ -2999,16 +2999,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>4073</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>1823</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>3244</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>9140</v>
       </c>
     </row>
     <row r="16">
@@ -4035,16 +4035,16 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>0</v>
+        <v>9294</v>
       </c>
       <c r="C15" t="n">
-        <v>0</v>
+        <v>4598</v>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>7289</v>
       </c>
       <c r="E15" t="n">
-        <v>0</v>
+        <v>21181</v>
       </c>
     </row>
     <row r="16">
@@ -5263,16 +5263,16 @@
         <v>3309</v>
       </c>
       <c r="F15" t="n">
-        <v>0</v>
+        <v>4073</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>1823</v>
       </c>
       <c r="H15" t="n">
-        <v>0</v>
+        <v>3244</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>9140</v>
       </c>
     </row>
     <row r="16">
@@ -6502,7 +6502,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6674,6 +6674,18 @@
       <c r="B14" t="inlineStr">
         <is>
           <t>C:\TRC\trc_engine\outputs\weekly\Weekly W13-2026.xlsx</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>W14</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>C:\TRC\trc_engine\outputs\weekly\Weekly W14-2026.xlsx</t>
         </is>
       </c>
     </row>
@@ -7967,7 +7979,7 @@
         <v>3762</v>
       </c>
       <c r="P9" s="7" t="n">
-        <v>0</v>
+        <v>4073</v>
       </c>
       <c r="Q9" s="7" t="n">
         <v>0</v>
@@ -8135,7 +8147,7 @@
         <v>1445</v>
       </c>
       <c r="P10" s="7" t="n">
-        <v>0</v>
+        <v>1823</v>
       </c>
       <c r="Q10" s="7" t="n">
         <v>0</v>
@@ -8303,7 +8315,7 @@
         <v>2211</v>
       </c>
       <c r="P11" s="7" t="n">
-        <v>0</v>
+        <v>3244</v>
       </c>
       <c r="Q11" s="7" t="n">
         <v>0</v>
@@ -8803,7 +8815,7 @@
         <v>7619</v>
       </c>
       <c r="P15" s="7" t="n">
-        <v>0</v>
+        <v>9294</v>
       </c>
       <c r="Q15" s="7" t="n">
         <v>0</v>
@@ -8971,7 +8983,7 @@
         <v>3146</v>
       </c>
       <c r="P16" s="7" t="n">
-        <v>0</v>
+        <v>4598</v>
       </c>
       <c r="Q16" s="7" t="n">
         <v>0</v>
@@ -9139,7 +9151,7 @@
         <v>4157</v>
       </c>
       <c r="P17" s="7" t="n">
-        <v>0</v>
+        <v>7289</v>
       </c>
       <c r="Q17" s="7" t="n">
         <v>0</v>

</xml_diff>